<commit_message>
Réponse 2 vague 4 : structure imposée sur 24 pages (rejet 10/10, reconstitution 11/11, taxation 3/8)
Chaque page : résumé des reproches du fisc, un sous-titre par point dans l'ordre
de son dernier rapport, carte rouge + popin du reproche détaillé, arguments,
documents par section. Cas de suppressions (89) et journées de paiements
fractionnés réembarqués. Nouveaux kinds liste/reproche/documents dans le rendu.
Pièces R2 à formules étendues ou créées (7 nouvelles).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YXeuvw5FcfiJESGdc5g8m6
</commit_message>
<xml_diff>
--- a/public/documents/pieces-reponse-2/R2-alcool-cuisine.xlsx
+++ b/public/documents/pieces-reponse-2/R2-alcool-cuisine.xlsx
@@ -11,6 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calcul" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Euros" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methode" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Euros_exercices" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prix_B1_B2_B3" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reserve_porto_ex1" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -550,9 +553,6 @@
       <c r="J4" t="n">
         <v>155.54</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -587,9 +587,6 @@
       <c r="J5" t="n">
         <v>74.06</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -624,9 +621,6 @@
       <c r="J6" t="n">
         <v>37.48</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -747,9 +741,6 @@
       <c r="J9" t="n">
         <v>11.32</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -784,9 +775,6 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -828,7 +816,7 @@
         <v>1.4</v>
       </c>
       <c r="M11" t="n">
-        <v>6.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="12">
@@ -864,9 +852,6 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -901,9 +886,6 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -916,6 +898,13 @@
       <c r="A16" t="inlineStr">
         <is>
           <t>Ravelin : le service retranche la part cuisine du volume unique des BIB sur les TROIS exercices ; l'annexe 7-1 (p.51) porte le ravelin sur l'exercice 1 (25 bouteilles, 1 875 cl ; ligne 'Fondue Jurassienne 372 x 10 = 3 720'). La premisse 'ex1 = 0 retranche' est donc fausse : supplement ravelin = 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Grand Marnier, exercice 3 : 9 bouteilles facturees (code 510090) dont 3 reprises par avoir sur la facture n° 526876 du 25/09/2024 : plafond net 6 bouteilles = 4,2 L (sans effet : demande 1,76 L).</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1867,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ce montant est l'effet sur le CA LIQUIDES reconstitue (TTC), avant application du coefficient liquides/solides et de la TVA par le service. Son exactitude par exercice suppose la communication des annexes 7-1 a 7-3 (prix unitaire reellement applique) et des annexes B des exercices 2023-2024 et 2024-2025, absentes du dossier.</t>
+          <t>Ce montant est l'effet sur le CA LIQUIDES reconstitue (TTC), avant l'abattement de 15 % et le coefficient liquides/solides appliques par le service (voir onglet Euros_exercices). Prix de l'annexe B1 appliques aux trois exercices (borne basse) ; la variante aux prix moyens de caisse de chaque exercice (annexes B1, B2, B3) figure a l'onglet Prix_B1_B2_B3. Le Grand Marnier n'a pas de prix de vente au verre en 2022-2023 (aucune vente) ; 6,50 EUR en 2023-2024 et 2024-2025.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1906,9 +1895,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1916,9 +1902,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1947,9 +1930,6 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1957,9 +1937,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -1974,9 +1951,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -1991,14 +1965,1176 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EUROS (onglet Euros). Effet sur le CA liquides reconstitue (TTC) = litres x 100 x (prix du verre / cl du verre), prix lus dans l'annexe B1 (2022-2023). Grand Marnier non chiffre faute de prix de vente au verre dans B1.</t>
-        </is>
+          <t>EUROS (onglets Euros, Euros_exercices, Prix_B1_B2_B3). Effet sur le CA liquides reconstitue (TTC) = litres x 100 x (prix du verre / cl du verre), prix de l'annexe B1 (2022-2023) appliques aux 3 exercices = 5 112,6 EUR hors Grand Marnier (borne basse). Variante aux prix moyens de caisse B1/B2/B3 : 5 411 EUR hors Grand Marnier, 5 925 EUR avec le Grand Marnier des exercices 2 et 3 (6,50 EUR le verre). Effet sur le total reconstitue : x 0,85 (abattement 15 %) x (1 + rapport liquides/solides) = 17 466 EUR TTC sur 3 exercices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RESERVE (onglet Reserve_porto_ex1). Le plafond porto de l'exercice 1 (16,5 L, 22 bouteilles) est inferieur aux 42 bouteilles de 75 cl facturees (31,5 L) : sans ce plafond, le supplement porto de l'exercice 1 serait de 14,99 L au lieu de 12,52 L (+2,47 L, +173 EUR). Le 72,68 L retenu est une borne basse ; la reserve n'est pas revendiquee.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Supplement a la carte par exercice (L, onglet Calcul colonnes H:J moins part menus O:Q) et conversion en euros aux prix de l'annexe B1 (2022-2023), puis effet sur le total reconstitue (abattement 15 % puis coefficient liquides/solides du service).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Alcool</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Supp. carte ex1 (L)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ex2</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ex3</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>3 ex</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Prix verre B1 (EUR)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>cl/verre</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>EUR par litre</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Euros ex1</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Euros ex2</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Euros ex3</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Euros 3 ex</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vin jaune</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>Calcul!H6-Calcul!O6</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>Calcul!I6-Calcul!P6</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>Calcul!J6-Calcul!Q6</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>SUM(B4:D4)</f>
+        <v/>
+      </c>
+      <c r="F4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4">
+        <f>F4/G4*100</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>B4*$H4</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>C4*$H4</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>D4*$H4</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>SUM(I4:K4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>Calcul!H8-Calcul!O8</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>Calcul!I8-Calcul!P8</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>Calcul!J8-Calcul!Q8</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>SUM(B5:D5)</f>
+        <v/>
+      </c>
+      <c r="F5" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <f>F5/G5*100</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>B5*$H5</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>C5*$H5</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>D5*$H5</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>SUM(I5:K5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bailey's (IVRESSE)</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>Calcul!H10-Calcul!O10</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>Calcul!I10-Calcul!P10</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>Calcul!J10-Calcul!Q10</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>SUM(B6:D6)</f>
+        <v/>
+      </c>
+      <c r="F6" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <f>F6/G6*100</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>B6*$H6</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>C6*$H6</f>
+        <v/>
+      </c>
+      <c r="K6">
+        <f>D6*$H6</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>SUM(I6:K6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Grand Marnier</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>Calcul!H11-Calcul!O11</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>Calcul!I11-Calcul!P11</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>Calcul!J11-Calcul!Q11</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SUM(B7:D7)</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>absent de B1 (aucun Grand Marnier vendu au verre en 2022-2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>SUM(B4:B7)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>SUM(C4:C7)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>SUM(D4:D7)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUM(E4:E7)</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>SUM(I4:I6)</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>SUM(J4:J6)</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>SUM(K4:K6)</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>SUM(L4:L6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Effet sur le total reconstitue du service (TTC) : euros liquides x (1 - 0,15) x (1 + rapport liquides/solides). Rapports 2,94 / 3,02 / 3,10 (proposition p. 52) ; facteurs 3,94 / 4,02 / 4,10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Exercice</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Euros liquides (B1)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Abattement 15 %</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Liquides apres abattement</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Rapport liquides/solides</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Facteur 1 + rapport</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Effet total reconstitue TTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2022-2023</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>I8</f>
+        <v/>
+      </c>
+      <c r="C12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D12">
+        <f>B12*(1-C12)</f>
+        <v/>
+      </c>
+      <c r="E12" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="F12">
+        <f>1+E12</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>D12*F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2023-2024</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>J8</f>
+        <v/>
+      </c>
+      <c r="C13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D13">
+        <f>B13*(1-C13)</f>
+        <v/>
+      </c>
+      <c r="E13" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="F13">
+        <f>1+E13</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>D13*F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2024-2025</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>K8</f>
+        <v/>
+      </c>
+      <c r="C14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D14">
+        <f>B14*(1-C14)</f>
+        <v/>
+      </c>
+      <c r="E14" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F14">
+        <f>1+E14</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>D14*F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL 3 exercices</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>SUM(B12:B14)</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>SUM(D12:D14)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>SUM(G12:G14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ordre de grandeur des droits (taux marginaux ; chiffrage exact dans les pages de taxation) : part liquides TTC a 20 %, part solides TTC a 10 %, IS 25 %, majoration 40 % (art. 1729).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>TTC</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>TVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Liquides (20 %)</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>D15</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>B19/1.2</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>B19-C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Solides (10 %)</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>G15-D15</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>B20/1.1</f>
+        <v/>
+      </c>
+      <c r="D20">
+        <f>B20-C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>B19+B20</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>C19+C20</f>
+        <v/>
+      </c>
+      <c r="D21">
+        <f>D19+D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>IS 25 % sur HT</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>C21*0.25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Majoration 40 % sur IS + TVA</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>(B22+D21)*0.4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Base distribuee (TTC) en moins, art. 109 : = total TTC</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Effet foyers aux taux effectifs 83,5 % / 73,2 % sur la moitie chacun (ordre de grandeur)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>B24/2*0.835+B24/2*0.732</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Variante : prix moyen de caisse de chaque exercice (annexes B1, B2, B3 : total TTC / quantite, lignes 'Vin jaune' ref 367, 'Porto' ref 9, 'Baileys'/'BAILEYS' ref 2096 et 2083, 'Grand Marnier' ref 2038). Le chiffre retenu dans la page reste 5 113 EUR (prix B1 sur les 3 exercices, borne basse).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Alcool</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Qte B1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Total TTC B1</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Prix moyen B1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Qte B2</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Total TTC B2</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Prix moyen B2</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Qte B3</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Total TTC B3</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Prix moyen B3</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>cl/verre</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Supp. ex1 (L)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Supp. ex2 (L)</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Supp. ex3 (L)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Euros ex1</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Euros ex2</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Euros ex3</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Euros 3 ex</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vin jaune</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1044</v>
+      </c>
+      <c r="D4">
+        <f>C4/B4</f>
+        <v/>
+      </c>
+      <c r="E4" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1284</v>
+      </c>
+      <c r="G4">
+        <f>F4/E4</f>
+        <v/>
+      </c>
+      <c r="H4" t="n">
+        <v>128</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1452</v>
+      </c>
+      <c r="J4">
+        <f>I4/H4</f>
+        <v/>
+      </c>
+      <c r="K4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L4">
+        <f>Euros_exercices!B4</f>
+        <v/>
+      </c>
+      <c r="M4">
+        <f>Euros_exercices!C4</f>
+        <v/>
+      </c>
+      <c r="N4">
+        <f>Euros_exercices!D4</f>
+        <v/>
+      </c>
+      <c r="O4">
+        <f>L4*100/$K4*D4</f>
+        <v/>
+      </c>
+      <c r="P4">
+        <f>M4*100/$K4*G4</f>
+        <v/>
+      </c>
+      <c r="Q4">
+        <f>N4*100/$K4*J4</f>
+        <v/>
+      </c>
+      <c r="R4">
+        <f>SUM(O4:Q4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>149.1</v>
+      </c>
+      <c r="D5">
+        <f>C5/B5</f>
+        <v/>
+      </c>
+      <c r="E5" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>226.8</v>
+      </c>
+      <c r="G5">
+        <f>F5/E5</f>
+        <v/>
+      </c>
+      <c r="H5" t="n">
+        <v>49</v>
+      </c>
+      <c r="I5" t="n">
+        <v>230.3</v>
+      </c>
+      <c r="J5">
+        <f>I5/H5</f>
+        <v/>
+      </c>
+      <c r="K5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <f>Euros_exercices!B5</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>Euros_exercices!C5</f>
+        <v/>
+      </c>
+      <c r="N5">
+        <f>Euros_exercices!D5</f>
+        <v/>
+      </c>
+      <c r="O5">
+        <f>L5*100/$K5*D5</f>
+        <v/>
+      </c>
+      <c r="P5">
+        <f>M5*100/$K5*G5</f>
+        <v/>
+      </c>
+      <c r="Q5">
+        <f>N5*100/$K5*J5</f>
+        <v/>
+      </c>
+      <c r="R5">
+        <f>SUM(O5:Q5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bailey's (IVRESSE)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6">
+        <f>C6/B6</f>
+        <v/>
+      </c>
+      <c r="E6" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="G6">
+        <f>F6/E6</f>
+        <v/>
+      </c>
+      <c r="H6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>52</v>
+      </c>
+      <c r="J6">
+        <f>I6/H6</f>
+        <v/>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <f>Euros_exercices!B6</f>
+        <v/>
+      </c>
+      <c r="M6">
+        <f>Euros_exercices!C6</f>
+        <v/>
+      </c>
+      <c r="N6">
+        <f>Euros_exercices!D6</f>
+        <v/>
+      </c>
+      <c r="O6">
+        <f>L6*100/$K6*D6</f>
+        <v/>
+      </c>
+      <c r="P6">
+        <f>M6*100/$K6*G6</f>
+        <v/>
+      </c>
+      <c r="Q6">
+        <f>N6*100/$K6*J6</f>
+        <v/>
+      </c>
+      <c r="R6">
+        <f>SUM(O6:Q6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Grand Marnier</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>aucune vente</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G7">
+        <f>F7/E7</f>
+        <v/>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>26</v>
+      </c>
+      <c r="J7">
+        <f>I7/H7</f>
+        <v/>
+      </c>
+      <c r="K7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7">
+        <f>Euros_exercices!B7</f>
+        <v/>
+      </c>
+      <c r="M7">
+        <f>Euros_exercices!C7</f>
+        <v/>
+      </c>
+      <c r="N7">
+        <f>Euros_exercices!D7</f>
+        <v/>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <f>M7*100/$K7*G7</f>
+        <v/>
+      </c>
+      <c r="Q7">
+        <f>N7*100/$K7*J7</f>
+        <v/>
+      </c>
+      <c r="R7">
+        <f>SUM(O7:Q7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL hors Grand Marnier</t>
+        </is>
+      </c>
+      <c r="O8">
+        <f>SUM(O4:O6)</f>
+        <v/>
+      </c>
+      <c r="P8">
+        <f>SUM(P4:P6)</f>
+        <v/>
+      </c>
+      <c r="Q8">
+        <f>SUM(Q4:Q6)</f>
+        <v/>
+      </c>
+      <c r="R8">
+        <f>SUM(R4:R6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL avec Grand Marnier ex2 et ex3</t>
+        </is>
+      </c>
+      <c r="O9">
+        <f>SUM(O4:O7)</f>
+        <v/>
+      </c>
+      <c r="P9">
+        <f>SUM(P4:P7)</f>
+        <v/>
+      </c>
+      <c r="Q9">
+        <f>SUM(Q4:Q7)</f>
+        <v/>
+      </c>
+      <c r="R9">
+        <f>SUM(R4:R7)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Reserve non revendiquee : le plafond porto de l'exercice 1 (16,5 L = 22 bouteilles) est inferieur aux achats factures FCBS de l'exercice 1 (codes 580018, 520077, 580019 : 42 bouteilles de 75 cl). Le 72,68 L retenu est donc une borne basse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bouteilles facturees ex1 (75 cl)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>42</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>factures FCBS 08/04/2022 a 24/03/2023, codes 580018 (19 + 21), 520077 (1), 580019 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Achats ex1 (L)</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>B4*0.75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plafond retenu dans Sources!K8 (L)</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>Sources!K8</f>
+        <v/>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>22 bouteilles seulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Demande ex1 carte + menus (L)</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>Calcul!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Deja retranche ex1 (L)</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>Sources!H8</f>
+        <v/>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>repere G, 398 cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Supplement ex1 retenu (L)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>Calcul!H8</f>
+        <v/>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>plafonne a 16,5 L</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Supplement ex1 sans plafond (L)</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>MAX(0,B7-B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ecart en litres</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>B10-B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ecart en euros (prix B1, 4,20 EUR / 6 cl)</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>B11*100*(4.2/6)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>